<commit_message>
Add analysis notebooks, figures and tables (H1-H3, theory applications)
- 01 stylized facts, 02 applied theory (offer curves, RCA, Grubel-Lloyd, PE)
- 03 ARDL bounds test (H1) with diagnostics, robust SEs, CUSUM
- 04 NARDL asymmetry (H2), 05 benchmark test, rolling elasticity, monthly LPs
- 06 supply vs demand shocks (H3) with Baumeister-Hamilton and Kanzig shocks
- Fix: RBI Table 32 duplicated FY1990-97 rows dropped; duplicate-block check added

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QxW88RBdwWvQZsaX3riENN
</commit_message>
<xml_diff>
--- a/data/processed/final_dataset.xlsx
+++ b/data/processed/final_dataset.xlsx
@@ -24727,18 +24727,6 @@
       <c r="AC32">
         <v>-5927.3</v>
       </c>
-      <c r="AD32">
-        <v>32</v>
-      </c>
-      <c r="AE32">
-        <v>100</v>
-      </c>
-      <c r="AF32">
-        <v>74</v>
-      </c>
-      <c r="AG32">
-        <v>9</v>
-      </c>
       <c r="AH32">
         <v>17.9428</v>
       </c>
@@ -24855,18 +24843,6 @@
       <c r="AC33">
         <v>-1545.1</v>
       </c>
-      <c r="AD33">
-        <v>32</v>
-      </c>
-      <c r="AE33">
-        <v>104</v>
-      </c>
-      <c r="AF33">
-        <v>79</v>
-      </c>
-      <c r="AG33">
-        <v>7</v>
-      </c>
       <c r="AH33">
         <v>24.4737</v>
       </c>
@@ -24983,18 +24959,6 @@
       <c r="AC34">
         <v>-3344.4</v>
       </c>
-      <c r="AD34">
-        <v>33</v>
-      </c>
-      <c r="AE34">
-        <v>109</v>
-      </c>
-      <c r="AF34">
-        <v>82</v>
-      </c>
-      <c r="AG34">
-        <v>7</v>
-      </c>
       <c r="AH34">
         <v>30.6488</v>
       </c>
@@ -25111,18 +25075,6 @@
       <c r="AC35">
         <v>-1067.9</v>
       </c>
-      <c r="AD35">
-        <v>33</v>
-      </c>
-      <c r="AE35">
-        <v>118</v>
-      </c>
-      <c r="AF35">
-        <v>90</v>
-      </c>
-      <c r="AG35">
-        <v>8</v>
-      </c>
       <c r="AH35">
         <v>31.3655</v>
       </c>
@@ -25254,18 +25206,6 @@
       <c r="AC36">
         <v>-2323.8</v>
       </c>
-      <c r="AD36">
-        <v>34</v>
-      </c>
-      <c r="AE36">
-        <v>123</v>
-      </c>
-      <c r="AF36">
-        <v>96</v>
-      </c>
-      <c r="AG36">
-        <v>9</v>
-      </c>
       <c r="AH36">
         <v>31.3986</v>
       </c>
@@ -25400,18 +25340,6 @@
       <c r="AC37">
         <v>-4880.4</v>
       </c>
-      <c r="AD37">
-        <v>32</v>
-      </c>
-      <c r="AE37">
-        <v>125</v>
-      </c>
-      <c r="AF37">
-        <v>99</v>
-      </c>
-      <c r="AG37">
-        <v>13</v>
-      </c>
       <c r="AH37">
         <v>33.4498</v>
       </c>
@@ -25546,18 +25474,6 @@
       <c r="AC38">
         <v>-5662.7</v>
       </c>
-      <c r="AD38">
-        <v>32</v>
-      </c>
-      <c r="AE38">
-        <v>141</v>
-      </c>
-      <c r="AF38">
-        <v>112</v>
-      </c>
-      <c r="AG38">
-        <v>18</v>
-      </c>
       <c r="AH38">
         <v>35.4999</v>
       </c>
@@ -25691,18 +25607,6 @@
       </c>
       <c r="AC39">
         <v>-6478</v>
-      </c>
-      <c r="AD39">
-        <v>32</v>
-      </c>
-      <c r="AE39">
-        <v>150</v>
-      </c>
-      <c r="AF39">
-        <v>122</v>
-      </c>
-      <c r="AG39">
-        <v>22</v>
       </c>
       <c r="AH39">
         <v>37.1648</v>

</xml_diff>